<commit_message>
fix(participant export): add the missing format when the list overflows the first page
</commit_message>
<xml_diff>
--- a/backend/src/modules/exports/templates/Form 12 - Registro de participantes v17ago23.xlsx
+++ b/backend/src/modules/exports/templates/Form 12 - Registro de participantes v17ago23.xlsx
@@ -83,10 +83,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,6 +136,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -196,61 +205,65 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -336,9 +349,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>914040</xdr:colOff>
+      <xdr:colOff>913680</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>314280</xdr:rowOff>
+      <xdr:rowOff>313920</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -347,8 +360,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6256080" y="744840"/>
-          <a:ext cx="860760" cy="283680"/>
+          <a:off x="6258600" y="744840"/>
+          <a:ext cx="860400" cy="283320"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst>
@@ -413,9 +426,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>677880</xdr:colOff>
+      <xdr:colOff>677520</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>373320</xdr:rowOff>
+      <xdr:rowOff>372960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -429,7 +442,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="76320" y="45720"/>
-          <a:ext cx="6804360" cy="660960"/>
+          <a:ext cx="6806520" cy="660600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -624,411 +637,417 @@
   <dimension ref="A1:I35"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="6.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="6.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.78"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="H5" s="7" t="s">
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="H5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="8"/>
+      <c r="I5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="H6" s="7" t="s">
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="H6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="8"/>
+      <c r="I6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9" t="s">
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="10" t="s">
+      <c r="F10" s="10"/>
+      <c r="G10" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I10" s="9" t="s">
+      <c r="I10" s="10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9" t="s">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="10"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="n">
+      <c r="A17" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="n">
+      <c r="A19" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="n">
+      <c r="A21" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="n">
+      <c r="A24" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="n">
+      <c r="A25" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="n">
+      <c r="A26" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="n">
+      <c r="A27" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="n">
+      <c r="A28" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="n">
+      <c r="A29" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B29" s="6"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="n">
+      <c r="A30" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="n">
+      <c r="A31" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="14" t="n">
+        <f aca="false">COUNTIF(E12:E31,"X")</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <f aca="false">COUNTIF(F12:F31,"X")</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="7"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="0" t="s">
+      <c r="C35" s="1" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>